<commit_message>
Migrate maps from Google Maps to Leaflet/OSM, secure Razorpay modal overlays, and fix registration redirects
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/E2E_Test_Report.xlsx
+++ b/Vulnerability Test Results/E2E_Test_Report.xlsx
@@ -17,7 +17,7 @@
     <t>JobNow Platform — Selenium E2E Test Report</t>
   </si>
   <si>
-    <t>Target: https://jobnow.dailywage.workers.dev  |  Run Date: 11/6/2026, 9:12:04 pm  |  Total: 43  ✅ PASS: 42  ❌ FAIL: 0  ⚠️ SKIP: 1</t>
+    <t>Target: https://jobnow.dailywage.workers.dev  |  Run Date: 13/6/2026, 12:04:21 am  |  Total: 43  ✅ PASS: 42  ❌ FAIL: 0  ⚠️ SKIP: 1</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -71,7 +71,7 @@
     <t/>
   </si>
   <si>
-    <t>9:07:12 pm</t>
+    <t>11:59:21 pm</t>
   </si>
   <si>
     <t>TC-02</t>
@@ -89,7 +89,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/welcome</t>
   </si>
   <si>
-    <t>9:07:16 pm</t>
+    <t>11:59:24 pm</t>
   </si>
   <si>
     <t>TC-03</t>
@@ -107,7 +107,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/login-choice</t>
   </si>
   <si>
-    <t>9:07:19 pm</t>
+    <t>11:59:27 pm</t>
   </si>
   <si>
     <t>TC-04</t>
@@ -125,7 +125,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/auth-choice?role=worker</t>
   </si>
   <si>
-    <t>9:07:22 pm</t>
+    <t>11:59:31 pm</t>
   </si>
   <si>
     <t>TC-05</t>
@@ -143,7 +143,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/login?role=worker</t>
   </si>
   <si>
-    <t>9:07:26 pm</t>
+    <t>11:59:34 pm</t>
   </si>
   <si>
     <t>TC-06</t>
@@ -161,7 +161,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/login?role=contractor</t>
   </si>
   <si>
-    <t>9:07:29 pm</t>
+    <t>11:59:38 pm</t>
   </si>
   <si>
     <t>TC-07</t>
@@ -179,7 +179,7 @@
     <t>Phone: true, Password: true</t>
   </si>
   <si>
-    <t>9:07:34 pm</t>
+    <t>11:59:43 pm</t>
   </si>
   <si>
     <t>TC-08</t>
@@ -200,7 +200,7 @@
     <t>Final URL: https://jobnow.dailywage.workers.dev/worker</t>
   </si>
   <si>
-    <t>9:07:47 pm</t>
+    <t>11:59:56 pm</t>
   </si>
   <si>
     <t>TC-09</t>
@@ -215,10 +215,10 @@
     <t>Dashboard has visible content</t>
   </si>
   <si>
-    <t>URL: https://jobnow.dailywage.workers.dev/worker, Content length: 806</t>
-  </si>
-  <si>
-    <t>9:07:49 pm</t>
+    <t>URL: https://jobnow.dailywage.workers.dev/worker, Content length: 926</t>
+  </si>
+  <si>
+    <t>11:59:58 pm</t>
   </si>
   <si>
     <t>TC-10</t>
@@ -236,7 +236,7 @@
     <t>Final URL: https://jobnow.dailywage.workers.dev/login?role=worker</t>
   </si>
   <si>
-    <t>9:08:09 pm</t>
+    <t>12:00:18 am</t>
   </si>
   <si>
     <t>TC-11</t>
@@ -248,7 +248,7 @@
     <t>Login with non-existent phone</t>
   </si>
   <si>
-    <t>9:08:55 pm</t>
+    <t>12:01:06 am</t>
   </si>
   <si>
     <t>TC-12</t>
@@ -269,7 +269,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/worker</t>
   </si>
   <si>
-    <t>9:09:07 pm</t>
+    <t>12:01:19 am</t>
   </si>
   <si>
     <t>TC-13</t>
@@ -287,7 +287,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/worker/jobs</t>
   </si>
   <si>
-    <t>9:09:11 pm</t>
+    <t>12:01:22 am</t>
   </si>
   <si>
     <t>TC-14</t>
@@ -305,7 +305,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/worker/profile</t>
   </si>
   <si>
-    <t>9:09:14 pm</t>
+    <t>12:01:26 am</t>
   </si>
   <si>
     <t>TC-15</t>
@@ -323,7 +323,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/worker/notifications</t>
   </si>
   <si>
-    <t>9:09:18 pm</t>
+    <t>12:01:29 am</t>
   </si>
   <si>
     <t>TC-16</t>
@@ -341,7 +341,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/worker/messages</t>
   </si>
   <si>
-    <t>9:09:21 pm</t>
+    <t>12:01:33 am</t>
   </si>
   <si>
     <t>TC-17</t>
@@ -359,7 +359,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/worker/earnings</t>
   </si>
   <si>
-    <t>9:09:24 pm</t>
+    <t>12:01:36 am</t>
   </si>
   <si>
     <t>TC-18</t>
@@ -377,7 +377,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/worker/settings</t>
   </si>
   <si>
-    <t>9:09:28 pm</t>
+    <t>12:01:39 am</t>
   </si>
   <si>
     <t>TC-19</t>
@@ -395,7 +395,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/worker/accepted</t>
   </si>
   <si>
-    <t>9:09:31 pm</t>
+    <t>12:01:43 am</t>
   </si>
   <si>
     <t>TC-20</t>
@@ -413,7 +413,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/worker/history</t>
   </si>
   <si>
-    <t>9:09:35 pm</t>
+    <t>12:01:46 am</t>
   </si>
   <si>
     <t>TC-21</t>
@@ -428,7 +428,7 @@
     <t>Redirected away from contractor area</t>
   </si>
   <si>
-    <t>9:09:38 pm</t>
+    <t>12:01:50 am</t>
   </si>
   <si>
     <t>TC-22</t>
@@ -446,7 +446,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/worker/help</t>
   </si>
   <si>
-    <t>9:09:41 pm</t>
+    <t>12:01:53 am</t>
   </si>
   <si>
     <t>TC-23</t>
@@ -467,7 +467,7 @@
     <t>Final URL: https://jobnow.dailywage.workers.dev/contractor</t>
   </si>
   <si>
-    <t>9:10:01 pm</t>
+    <t>12:02:14 am</t>
   </si>
   <si>
     <t>TC-24</t>
@@ -497,7 +497,7 @@
     <t>Final URL: https://jobnow.dailywage.workers.dev/login?role=contractor</t>
   </si>
   <si>
-    <t>9:10:21 pm</t>
+    <t>12:02:34 am</t>
   </si>
   <si>
     <t>TC-26</t>
@@ -515,7 +515,7 @@
     <t>Contractor dashboard accessible</t>
   </si>
   <si>
-    <t>9:10:33 pm</t>
+    <t>12:02:47 am</t>
   </si>
   <si>
     <t>TC-27</t>
@@ -533,7 +533,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/contractor/post</t>
   </si>
   <si>
-    <t>9:10:37 pm</t>
+    <t>12:02:51 am</t>
   </si>
   <si>
     <t>TC-28</t>
@@ -551,7 +551,7 @@
     <t>Input count: 8</t>
   </si>
   <si>
-    <t>9:10:42 pm</t>
+    <t>12:02:56 am</t>
   </si>
   <si>
     <t>TC-29</t>
@@ -569,7 +569,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/contractor/applications</t>
   </si>
   <si>
-    <t>9:10:45 pm</t>
+    <t>12:03:00 am</t>
   </si>
   <si>
     <t>TC-30</t>
@@ -587,7 +587,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/contractor/active</t>
   </si>
   <si>
-    <t>9:10:49 pm</t>
+    <t>12:03:03 am</t>
   </si>
   <si>
     <t>TC-31</t>
@@ -605,7 +605,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/contractor/payments</t>
   </si>
   <si>
-    <t>9:10:52 pm</t>
+    <t>12:03:07 am</t>
   </si>
   <si>
     <t>TC-32</t>
@@ -623,7 +623,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/contractor/analytics</t>
   </si>
   <si>
-    <t>9:10:55 pm</t>
+    <t>12:03:10 am</t>
   </si>
   <si>
     <t>TC-33</t>
@@ -638,7 +638,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/contractor/messages</t>
   </si>
   <si>
-    <t>9:10:59 pm</t>
+    <t>12:03:14 am</t>
   </si>
   <si>
     <t>TC-34</t>
@@ -653,7 +653,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/contractor/profile</t>
   </si>
   <si>
-    <t>9:11:02 pm</t>
+    <t>12:03:17 am</t>
   </si>
   <si>
     <t>TC-35</t>
@@ -668,7 +668,7 @@
     <t>Redirected away from worker area</t>
   </si>
   <si>
-    <t>9:11:06 pm</t>
+    <t>12:03:21 am</t>
   </si>
   <si>
     <t>TC-36</t>
@@ -686,7 +686,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/contractor/workers</t>
   </si>
   <si>
-    <t>9:11:09 pm</t>
+    <t>12:03:25 am</t>
   </si>
   <si>
     <t>TC-37</t>
@@ -701,7 +701,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/contractor/settings</t>
   </si>
   <si>
-    <t>9:11:12 pm</t>
+    <t>12:03:28 am</t>
   </si>
   <si>
     <t>TC-38</t>
@@ -719,7 +719,7 @@
     <t>Redirected to login/welcome</t>
   </si>
   <si>
-    <t>9:11:24 pm</t>
+    <t>12:03:40 am</t>
   </si>
   <si>
     <t>TC-39</t>
@@ -731,7 +731,7 @@
     <t>Access /contractor without login</t>
   </si>
   <si>
-    <t>9:11:28 pm</t>
+    <t>12:03:43 am</t>
   </si>
   <si>
     <t>TC-40</t>
@@ -749,7 +749,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/forgot-password?role=worker</t>
   </si>
   <si>
-    <t>9:11:31 pm</t>
+    <t>12:03:47 am</t>
   </si>
   <si>
     <t>TC-41</t>
@@ -767,7 +767,7 @@
     <t>URL: https://jobnow.dailywage.workers.dev/register?role=worker</t>
   </si>
   <si>
-    <t>9:11:34 pm</t>
+    <t>12:03:50 am</t>
   </si>
   <si>
     <t>TC-42</t>
@@ -782,7 +782,7 @@
     <t>Job listings page loads</t>
   </si>
   <si>
-    <t>9:11:52 pm</t>
+    <t>12:04:09 am</t>
   </si>
   <si>
     <t>TC-43</t>
@@ -803,7 +803,7 @@
     <t>SKIP</t>
   </si>
   <si>
-    <t>9:12:04 pm</t>
+    <t>12:04:20 am</t>
   </si>
   <si>
     <t>JobNow E2E Test Summary</t>
@@ -821,7 +821,7 @@
     <t>Test Run Date</t>
   </si>
   <si>
-    <t>11/6/2026, 9:12:04 pm</t>
+    <t>13/6/2026, 12:04:21 am</t>
   </si>
   <si>
     <t>Total Test Cases</t>

</xml_diff>